<commit_message>
chore: refresh Phase 1A workbook artifacts
Records content-equivalent workbook saves whose only worksheet delta is regenerated protection hash and salt metadata.
</commit_message>
<xml_diff>
--- a/outputs/01a04d4d-b17c-7212-9796-f7f88d59062b/Phase-1A-multi-HSP-presentation-demo.xlsx
+++ b/outputs/01a04d4d-b17c-7212-9796-f7f88d59062b/Phase-1A-multi-HSP-presentation-demo.xlsx
@@ -1309,7 +1309,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="21b6KXjfE5pvRZk68eHCMKxaBpXF4fLFHXK/f4ovKDUqmeG7JzHBDk7tysUZr5PTTfz0fu0DXDylULm3LFDMGQ==" saltValue="puZ2hJVblpYAYU+Ov4La4A==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="NETuz4SeqHzmTerlU+ettMQ0LmIBaYxf38oZGw4APuopqNhf9DWxu8dWN1OrcvW7kkvMRPyYDg3lOaWkxUoCtQ==" saltValue="2LGhuupyPNHrYbXgmZoLPA==" spinCount="100000"/>
   <mergeCells count="9">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B7:E7"/>
@@ -1480,7 +1480,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="50ZMgbTaEIhyr+7VvlIY8sJTI1Wghfib9PucVitYcMOta4qKTIJO9MBXDeWgebZnbMmZjw4evKqNm2uY6x/91w==" saltValue="bYhQM2v9WTSBQmqUnAlbng==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="t2mQ6+mXjlPpyYThci56ThAHxsQ7RpUINO4MQ9kHT0ZNTCxTXsWK96qoc2r//L8Lrv9t0K80NKT2LpXz1sqnpA==" saltValue="IoEx5N3TK9G10xKIBnBXbA==" spinCount="100000"/>
   <mergeCells count="3">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C9:G9"/>
@@ -1666,7 +1666,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="n9dtqwQxD6vcZ1wknDx/zjDOZnen9pWi0ncEigS85RFuyZtc953LRgJJIboBfjJU/RRCuMK6HBQC+CaJaRG+4Q==" saltValue="lcz2E4mKJIEOGqMWUkBdKw==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="yh2SQsldqGuBwljLcia3xcIt6Pry9F7ogCGVHwF8uFy0gXwmei7MFzBd1EWvg8L09NDm0b2bAjjvPO+bm3n+nw==" saltValue="8kDOv3yAhp3mstqO4W+F7g==" spinCount="100000"/>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
@@ -2154,7 +2154,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="evTap1ABxdSk0jYEN6yrStEKgTkDpDmFDLwLAJf2+0OigA3ISwKbZ4B3tXPzTr0+f2DI6jY+uCKoNUMZp6Sg+Q==" saltValue="P4jxPt+1XEsHimOkWAWkZQ==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="EPprYwwJX7QEutlsRbDL3vs6cz4ktpXxAlHJ7E11volnW3Jw8JciNVuclK3RIkcWINrzrYdUqhywW5Ch31hPpQ==" saltValue="84FozUpG9B5v5jH5zFGY/Q==" spinCount="100000"/>
   <mergeCells count="9">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A7:G7"/>
@@ -2506,7 +2506,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="mIHf9n+fLCRau74gPgVnx8fXdZ4HQBphFkW2Pn5eXt8iWpt/6PsKjAjoT+kGpUmSlkQHw7ZcfA5CLmk+AO55EA==" saltValue="B5PDVY2k3zIHCQl/vXbTOg==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="ENcJt84QDPNltG7wsz4AsDd9lcckNfi45NJeiDQOE45sf7rH/N3yR9MG3e4F5o3/F8e7epa/w8xo21bVczi2jQ==" saltValue="3Aq5oWtvm1TlmVTr8Jp0hQ==" spinCount="100000"/>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
@@ -2687,7 +2687,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="LBhFG5DmX4iy5zgUEF+ofgGlL6T6xcsCTbO68wuDxfsJJq2fFBhEd1lMmDAHuGMQuI03Rf7eQFOjOStF5C9nNA==" saltValue="lsAtcOrnXXCZVR0qivdmRA==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="9xBJArpS4aOCsmrsGH8o0EdyMQy8qBgHz2ltollVTO2a/aWEF2eqrMwjjJMlpVT0Jtpi/Xb3cTtUsw6AOnND/Q==" saltValue="oEylLSRGpOSyu4LMULDCmg==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="2">
@@ -3087,7 +3087,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="Wm22Budfobr/uNT3MRTSi6HgaxiT98M4FSBgokK34IskAQkOm5Dne2rV4pOkfivCq6TRVQmkmYhj59tbyP7kTA==" saltValue="DUkPBTpXpk20ShkrCZggaw==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="N16K9BKtoHJcxPJznZboOqwkjtVRKRih9Iv6zX+6SyER0Ehhve6jVZREaImhk5flQTKVWyNo8WbiEun0AHvs9w==" saltValue="JaLg2ccwHZF2AdtF6rrcmg==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
@@ -3207,7 +3207,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="C6HEJTI6n4Xpf9BgBSC4dR9ZBsXTWfBUv3eaC3O6j8AriE3AS3eqFhAWsfW/AZGTLf19jgaJsfOzIadgnmq+MA==" saltValue="ax+bkYERWNaXPCc8UBqVfQ==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="zK6r34oe4pK4dQVI3INSXzcLKsip989WgszTOUuxzJ5H+g/ncmik6gloncSSeukeIcKKE2XDk9jj+bXD+Lea0A==" saltValue="7rwRt+n6GJLEeyIZ4XmjkA==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
@@ -3278,7 +3278,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="AddWSNHFuKg2HsiEAcU7vtjFcgvHckr2y15OoVmebKzBMa8r24UkXKdYFX8Ym2OfbsIW3BMYwUmprAFWivrwUg==" saltValue="dL3EqujYeEgMyNVzJiycSQ==" spinCount="100000"/>
+  <sheetProtection sheet="1" selectUnlockedCells="1" algorithmName="SHA-512" hashValue="8hmXp2pb6gOwib5v3/Gw4+RMxhA92oDrchEoOqWPpBoSIkS0FCP10lchuV04I8a15fi9XKuqQaUm5FXJ6tWCag==" saltValue="UwtQt6irlUQaUtIPDKhClg==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">

</xml_diff>